<commit_message>
rename overallKPI to cycleKPI
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_lat.xlsx
+++ b/src/config/kpi_as_lat.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/config/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033D4CE4-1EB1-E140-AC93-796B4A7B4BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E0C5569-E408-5749-B405-27354103734B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="params" sheetId="1" r:id="rId1"/>
     <sheet name="graphSpec" sheetId="2" r:id="rId2"/>
     <sheet name="KPI" sheetId="3" r:id="rId3"/>
-    <sheet name="overallKPI" sheetId="6" r:id="rId4"/>
+    <sheet name="cycleKPI" sheetId="6" r:id="rId4"/>
     <sheet name="markerShapes" sheetId="4" r:id="rId5"/>
     <sheet name="lineColors" sheetId="5" r:id="rId6"/>
   </sheets>

</xml_diff>

<commit_message>
migrate vbRcSignals to long/lat_kpi excel and clean legacy comments
</commit_message>
<xml_diff>
--- a/src/config/kpi_as_lat.xlsx
+++ b/src/config/kpi_as_lat.xlsx
@@ -8,24 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wangjianhai/02_ADAS/01_repo/01_Tools/01_kpi_extractor/python/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E0C5569-E408-5749-B405-27354103734B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163D1C0A-35DE-2F44-9F23-D19AE9841531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="params" sheetId="1" r:id="rId1"/>
-    <sheet name="graphSpec" sheetId="2" r:id="rId2"/>
-    <sheet name="KPI" sheetId="3" r:id="rId3"/>
-    <sheet name="cycleKPI" sheetId="6" r:id="rId4"/>
-    <sheet name="markerShapes" sheetId="4" r:id="rId5"/>
-    <sheet name="lineColors" sheetId="5" r:id="rId6"/>
+    <sheet name="vbRcSignals" sheetId="7" r:id="rId1"/>
+    <sheet name="params" sheetId="1" r:id="rId2"/>
+    <sheet name="graphSpec" sheetId="2" r:id="rId3"/>
+    <sheet name="KPI" sheetId="3" r:id="rId4"/>
+    <sheet name="cycleKPI" sheetId="6" r:id="rId5"/>
+    <sheet name="markerShapes" sheetId="4" r:id="rId6"/>
+    <sheet name="lineColors" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="176">
   <si>
     <t>Parameter</t>
   </si>
@@ -397,14 +398,178 @@
   </si>
   <si>
     <t>feature</t>
+  </si>
+  <si>
+    <t>raster</t>
+  </si>
+  <si>
+    <t>synonym</t>
+  </si>
+  <si>
+    <t>genericName</t>
+  </si>
+  <si>
+    <t>imuFrame</t>
+  </si>
+  <si>
+    <t>acceleration[1]</t>
+  </si>
+  <si>
+    <t>latActAccel</t>
+  </si>
+  <si>
+    <t>acceleration[0]</t>
+  </si>
+  <si>
+    <t>longActAccel</t>
+  </si>
+  <si>
+    <t>vehicleIOActuationFeedback</t>
+  </si>
+  <si>
+    <t>speedESC</t>
+  </si>
+  <si>
+    <t>egoSpeed</t>
+  </si>
+  <si>
+    <t>throttle_value</t>
+  </si>
+  <si>
+    <t>throttleValue</t>
+  </si>
+  <si>
+    <t>vehicleIOstate</t>
+  </si>
+  <si>
+    <t>brake_pedal_pressed</t>
+  </si>
+  <si>
+    <t>brakePedalPressed</t>
+  </si>
+  <si>
+    <t>turnrate[2]</t>
+  </si>
+  <si>
+    <t>yawRate</t>
+  </si>
+  <si>
+    <t>vehicle_stopped</t>
+  </si>
+  <si>
+    <t>isVehStoppedNV</t>
+  </si>
+  <si>
+    <t>enum</t>
+  </si>
+  <si>
+    <t>DIStatus</t>
+  </si>
+  <si>
+    <t>active_safety_status/notices/LKA/intervention_status</t>
+  </si>
+  <si>
+    <t>lkaInterventionStatus</t>
+  </si>
+  <si>
+    <t>lane_support_system_debug</t>
+  </si>
+  <si>
+    <t>dtle_actuation_threshold</t>
+  </si>
+  <si>
+    <t>dtleTarget</t>
+  </si>
+  <si>
+    <t>current_DTLE</t>
+  </si>
+  <si>
+    <t>dtle</t>
+  </si>
+  <si>
+    <t>steering_wheel_torque</t>
+  </si>
+  <si>
+    <t>steerWheelTorque</t>
+  </si>
+  <si>
+    <t>rate_of_departure</t>
+  </si>
+  <si>
+    <t>rateOfDeparture</t>
+  </si>
+  <si>
+    <t>float_x000D_</t>
+  </si>
+  <si>
+    <t>lat_ctrl_curvature_actual</t>
+  </si>
+  <si>
+    <t>vehCurvature</t>
+  </si>
+  <si>
+    <t>lane_curvature</t>
+  </si>
+  <si>
+    <t>laneCurvature</t>
+  </si>
+  <si>
+    <t>lane_support_system_request</t>
+  </si>
+  <si>
+    <t>use_case</t>
+  </si>
+  <si>
+    <t>useCase</t>
+  </si>
+  <si>
+    <t>active_safety_status/notices/LKA/ready_left</t>
+  </si>
+  <si>
+    <t>lkaReadyLeft</t>
+  </si>
+  <si>
+    <t>active_safety_status/notices/LKA/ready_right</t>
+  </si>
+  <si>
+    <t>lkaReadyRight</t>
+  </si>
+  <si>
+    <t>active_safety_status/settings/LKA/actuation_precondition_blocked</t>
+  </si>
+  <si>
+    <t>lkaPrecondBlk</t>
+  </si>
+  <si>
+    <t>active_safety_status/settings/LKA/abort_any_active_events</t>
+  </si>
+  <si>
+    <t>lkaAbort</t>
+  </si>
+  <si>
+    <t>gpsFrame</t>
+  </si>
+  <si>
+    <t>latitude</t>
+  </si>
+  <si>
+    <t>longitude</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -432,8 +597,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -772,6 +938,330 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B475A55-00E3-6140-B3DA-E969C5DB794A}">
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="31.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" t="s">
+        <v>146</v>
+      </c>
+      <c r="C9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C10" t="s">
+        <v>150</v>
+      </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>148</v>
+      </c>
+      <c r="B11" t="s">
+        <v>151</v>
+      </c>
+      <c r="C11" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" t="s">
+        <v>153</v>
+      </c>
+      <c r="C12" t="s">
+        <v>154</v>
+      </c>
+      <c r="D12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>148</v>
+      </c>
+      <c r="B13" t="s">
+        <v>155</v>
+      </c>
+      <c r="C13" t="s">
+        <v>156</v>
+      </c>
+      <c r="D13" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B14" t="s">
+        <v>158</v>
+      </c>
+      <c r="C14" t="s">
+        <v>159</v>
+      </c>
+      <c r="D14" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>148</v>
+      </c>
+      <c r="B15" t="s">
+        <v>160</v>
+      </c>
+      <c r="C15" t="s">
+        <v>161</v>
+      </c>
+      <c r="D15" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>162</v>
+      </c>
+      <c r="B16" t="s">
+        <v>163</v>
+      </c>
+      <c r="C16" t="s">
+        <v>164</v>
+      </c>
+      <c r="D16" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>145</v>
+      </c>
+      <c r="B17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C17" t="s">
+        <v>166</v>
+      </c>
+      <c r="D17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>145</v>
+      </c>
+      <c r="B18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C18" t="s">
+        <v>168</v>
+      </c>
+      <c r="D18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>145</v>
+      </c>
+      <c r="B19" t="s">
+        <v>169</v>
+      </c>
+      <c r="C19" t="s">
+        <v>170</v>
+      </c>
+      <c r="D19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>145</v>
+      </c>
+      <c r="B20" t="s">
+        <v>171</v>
+      </c>
+      <c r="C20" t="s">
+        <v>172</v>
+      </c>
+      <c r="D20" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" t="s">
+        <v>174</v>
+      </c>
+      <c r="C21" t="s">
+        <v>174</v>
+      </c>
+      <c r="D21" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>173</v>
+      </c>
+      <c r="B22" t="s">
+        <v>175</v>
+      </c>
+      <c r="C22" t="s">
+        <v>175</v>
+      </c>
+      <c r="D22" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -824,7 +1314,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -989,7 +1479,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1213,7 +1703,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC7B1E6F-C944-5C4D-9BEC-4AD07790F7D1}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1303,7 +1793,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1361,7 +1851,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>